<commit_message>
Updated ML-framework code, improved scattering fitting and AFM analysis
</commit_message>
<xml_diff>
--- a/machine_learning/classification_models/input_data/pspeo_master.xlsx
+++ b/machine_learning/classification_models/input_data/pspeo_master.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">afm_grain</t>
   </si>
   <si>
-    <t xml:space="preserve">order_disorder</t>
+    <t xml:space="preserve">tri</t>
   </si>
   <si>
     <t xml:space="preserve">I_A_AC</t>
@@ -776,7 +776,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I203"/>
-  <sheetFormatPr defaultColWidth="8.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="2.26"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -803,7 +806,7 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="0" t="s">
         <v>8</v>
       </c>
     </row>
@@ -832,7 +835,7 @@
       <c r="H2" s="1" t="n">
         <v>0.0048</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -861,8 +864,8 @@
       <c r="H3" s="1" t="n">
         <v>0.0047</v>
       </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
+      <c r="I3" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -890,8 +893,8 @@
       <c r="H4" s="1" t="n">
         <v>0.0534</v>
       </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
+      <c r="I4" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -919,8 +922,8 @@
       <c r="H5" s="1" t="n">
         <v>0.0425</v>
       </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
+      <c r="I5" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -948,8 +951,8 @@
       <c r="H6" s="1" t="n">
         <v>0.0244</v>
       </c>
-      <c r="I6" s="1" t="n">
-        <v>0</v>
+      <c r="I6" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -977,8 +980,8 @@
       <c r="H7" s="1" t="n">
         <v>0.1137</v>
       </c>
-      <c r="I7" s="1" t="n">
-        <v>1</v>
+      <c r="I7" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1006,8 +1009,8 @@
       <c r="H8" s="1" t="n">
         <v>0.0907</v>
       </c>
-      <c r="I8" s="1" t="n">
-        <v>1</v>
+      <c r="I8" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1035,8 +1038,8 @@
       <c r="H9" s="1" t="n">
         <v>0.1287</v>
       </c>
-      <c r="I9" s="1" t="n">
-        <v>1</v>
+      <c r="I9" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1064,8 +1067,8 @@
       <c r="H10" s="1" t="n">
         <v>0.0617</v>
       </c>
-      <c r="I10" s="1" t="n">
-        <v>1</v>
+      <c r="I10" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1093,8 +1096,8 @@
       <c r="H11" s="1" t="n">
         <v>0.3226</v>
       </c>
-      <c r="I11" s="1" t="n">
-        <v>1</v>
+      <c r="I11" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,8 +1125,8 @@
       <c r="H12" s="1" t="n">
         <v>0.0892</v>
       </c>
-      <c r="I12" s="1" t="n">
-        <v>1</v>
+      <c r="I12" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1151,8 +1154,8 @@
       <c r="H13" s="1" t="n">
         <v>0.0795</v>
       </c>
-      <c r="I13" s="1" t="n">
-        <v>1</v>
+      <c r="I13" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1180,8 +1183,8 @@
       <c r="H14" s="1" t="n">
         <v>0.0987</v>
       </c>
-      <c r="I14" s="1" t="n">
-        <v>1</v>
+      <c r="I14" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1209,8 +1212,8 @@
       <c r="H15" s="1" t="n">
         <v>0.2132</v>
       </c>
-      <c r="I15" s="1" t="n">
-        <v>1</v>
+      <c r="I15" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1238,8 +1241,8 @@
       <c r="H16" s="1" t="n">
         <v>0.111</v>
       </c>
-      <c r="I16" s="1" t="n">
-        <v>1</v>
+      <c r="I16" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1267,8 +1270,8 @@
       <c r="H17" s="1" t="n">
         <v>0.1188</v>
       </c>
-      <c r="I17" s="1" t="n">
-        <v>1</v>
+      <c r="I17" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1296,8 +1299,8 @@
       <c r="H18" s="1" t="n">
         <v>0.2669</v>
       </c>
-      <c r="I18" s="1" t="n">
-        <v>1</v>
+      <c r="I18" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1325,8 +1328,8 @@
       <c r="H19" s="1" t="n">
         <v>0.2157</v>
       </c>
-      <c r="I19" s="1" t="n">
-        <v>1</v>
+      <c r="I19" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1354,8 +1357,8 @@
       <c r="H20" s="1" t="n">
         <v>0.1838</v>
       </c>
-      <c r="I20" s="1" t="n">
-        <v>1</v>
+      <c r="I20" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1383,8 +1386,8 @@
       <c r="H21" s="1" t="n">
         <v>0.2041</v>
       </c>
-      <c r="I21" s="1" t="n">
-        <v>1</v>
+      <c r="I21" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1412,8 +1415,8 @@
       <c r="H22" s="1" t="n">
         <v>0.1738</v>
       </c>
-      <c r="I22" s="1" t="n">
-        <v>1</v>
+      <c r="I22" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1441,8 +1444,8 @@
       <c r="H23" s="1" t="n">
         <v>0.2165</v>
       </c>
-      <c r="I23" s="1" t="n">
-        <v>1</v>
+      <c r="I23" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1470,8 +1473,8 @@
       <c r="H24" s="1" t="n">
         <v>0.3211</v>
       </c>
-      <c r="I24" s="1" t="n">
-        <v>1</v>
+      <c r="I24" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1499,8 +1502,8 @@
       <c r="H25" s="1" t="n">
         <v>0.233</v>
       </c>
-      <c r="I25" s="1" t="n">
-        <v>1</v>
+      <c r="I25" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1528,8 +1531,8 @@
       <c r="H26" s="1" t="n">
         <v>0.715</v>
       </c>
-      <c r="I26" s="1" t="n">
-        <v>1</v>
+      <c r="I26" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1557,7 +1560,7 @@
       <c r="H27" s="1" t="n">
         <v>0.0029</v>
       </c>
-      <c r="I27" s="1" t="n">
+      <c r="I27" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1586,8 +1589,8 @@
       <c r="H28" s="1" t="n">
         <v>0.0049</v>
       </c>
-      <c r="I28" s="1" t="n">
-        <v>0</v>
+      <c r="I28" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1615,8 +1618,8 @@
       <c r="H29" s="1" t="n">
         <v>0.0183</v>
       </c>
-      <c r="I29" s="1" t="n">
-        <v>0</v>
+      <c r="I29" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1644,8 +1647,8 @@
       <c r="H30" s="1" t="n">
         <v>0.0144</v>
       </c>
-      <c r="I30" s="1" t="n">
-        <v>0</v>
+      <c r="I30" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,8 +1676,8 @@
       <c r="H31" s="1" t="n">
         <v>0.0477</v>
       </c>
-      <c r="I31" s="1" t="n">
-        <v>0</v>
+      <c r="I31" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1702,8 +1705,8 @@
       <c r="H32" s="1" t="n">
         <v>0.1473</v>
       </c>
-      <c r="I32" s="1" t="n">
-        <v>1</v>
+      <c r="I32" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1731,8 +1734,8 @@
       <c r="H33" s="1" t="n">
         <v>0.1068</v>
       </c>
-      <c r="I33" s="1" t="n">
-        <v>1</v>
+      <c r="I33" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1760,8 +1763,8 @@
       <c r="H34" s="1" t="n">
         <v>0.066</v>
       </c>
-      <c r="I34" s="1" t="n">
-        <v>1</v>
+      <c r="I34" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1789,8 +1792,8 @@
       <c r="H35" s="1" t="n">
         <v>0.1334</v>
       </c>
-      <c r="I35" s="1" t="n">
-        <v>1</v>
+      <c r="I35" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1818,8 +1821,8 @@
       <c r="H36" s="1" t="n">
         <v>0.0698</v>
       </c>
-      <c r="I36" s="1" t="n">
-        <v>1</v>
+      <c r="I36" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,8 +1850,8 @@
       <c r="H37" s="1" t="n">
         <v>0.0932</v>
       </c>
-      <c r="I37" s="1" t="n">
-        <v>1</v>
+      <c r="I37" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1876,8 +1879,8 @@
       <c r="H38" s="1" t="n">
         <v>0.1233</v>
       </c>
-      <c r="I38" s="1" t="n">
-        <v>1</v>
+      <c r="I38" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1905,8 +1908,8 @@
       <c r="H39" s="1" t="n">
         <v>0.1492</v>
       </c>
-      <c r="I39" s="1" t="n">
-        <v>1</v>
+      <c r="I39" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1934,8 +1937,8 @@
       <c r="H40" s="1" t="n">
         <v>0.1048</v>
       </c>
-      <c r="I40" s="1" t="n">
-        <v>1</v>
+      <c r="I40" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1963,8 +1966,8 @@
       <c r="H41" s="1" t="n">
         <v>0.0795</v>
       </c>
-      <c r="I41" s="1" t="n">
-        <v>1</v>
+      <c r="I41" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1992,8 +1995,8 @@
       <c r="H42" s="1" t="n">
         <v>0.1302</v>
       </c>
-      <c r="I42" s="1" t="n">
-        <v>1</v>
+      <c r="I42" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2021,8 +2024,8 @@
       <c r="H43" s="1" t="n">
         <v>0.1078</v>
       </c>
-      <c r="I43" s="1" t="n">
-        <v>1</v>
+      <c r="I43" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2050,8 +2053,8 @@
       <c r="H44" s="1" t="n">
         <v>0.1004</v>
       </c>
-      <c r="I44" s="1" t="n">
-        <v>1</v>
+      <c r="I44" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2079,8 +2082,8 @@
       <c r="H45" s="1" t="n">
         <v>0.1656</v>
       </c>
-      <c r="I45" s="1" t="n">
-        <v>1</v>
+      <c r="I45" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2108,8 +2111,8 @@
       <c r="H46" s="1" t="n">
         <v>0.1026</v>
       </c>
-      <c r="I46" s="1" t="n">
-        <v>1</v>
+      <c r="I46" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2137,8 +2140,8 @@
       <c r="H47" s="1" t="n">
         <v>0.0895</v>
       </c>
-      <c r="I47" s="1" t="n">
-        <v>1</v>
+      <c r="I47" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2166,8 +2169,8 @@
       <c r="H48" s="1" t="n">
         <v>0.0833</v>
       </c>
-      <c r="I48" s="1" t="n">
-        <v>1</v>
+      <c r="I48" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2195,8 +2198,8 @@
       <c r="H49" s="1" t="n">
         <v>0.1417</v>
       </c>
-      <c r="I49" s="1" t="n">
-        <v>1</v>
+      <c r="I49" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2224,8 +2227,8 @@
       <c r="H50" s="1" t="n">
         <v>0.2062</v>
       </c>
-      <c r="I50" s="1" t="n">
-        <v>1</v>
+      <c r="I50" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2253,8 +2256,8 @@
       <c r="H51" s="1" t="n">
         <v>0.2381</v>
       </c>
-      <c r="I51" s="1" t="n">
-        <v>1</v>
+      <c r="I51" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,7 +2285,7 @@
       <c r="H52" s="1" t="n">
         <v>0.0035</v>
       </c>
-      <c r="I52" s="1" t="n">
+      <c r="I52" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2311,8 +2314,8 @@
       <c r="H53" s="1" t="n">
         <v>0.0069</v>
       </c>
-      <c r="I53" s="1" t="n">
-        <v>0</v>
+      <c r="I53" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2340,8 +2343,8 @@
       <c r="H54" s="1" t="n">
         <v>0.0289</v>
       </c>
-      <c r="I54" s="1" t="n">
-        <v>0</v>
+      <c r="I54" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2369,8 +2372,8 @@
       <c r="H55" s="1" t="n">
         <v>0.0532</v>
       </c>
-      <c r="I55" s="1" t="n">
-        <v>0</v>
+      <c r="I55" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2398,8 +2401,8 @@
       <c r="H56" s="1" t="n">
         <v>0.0372</v>
       </c>
-      <c r="I56" s="1" t="n">
-        <v>0</v>
+      <c r="I56" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2427,8 +2430,8 @@
       <c r="H57" s="1" t="n">
         <v>0.1171</v>
       </c>
-      <c r="I57" s="1" t="n">
-        <v>1</v>
+      <c r="I57" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2456,8 +2459,8 @@
       <c r="H58" s="1" t="n">
         <v>0.0598</v>
       </c>
-      <c r="I58" s="1" t="n">
-        <v>1</v>
+      <c r="I58" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2485,8 +2488,8 @@
       <c r="H59" s="1" t="n">
         <v>0.0649</v>
       </c>
-      <c r="I59" s="1" t="n">
-        <v>1</v>
+      <c r="I59" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2514,8 +2517,8 @@
       <c r="H60" s="1" t="n">
         <v>0.1736</v>
       </c>
-      <c r="I60" s="1" t="n">
-        <v>1</v>
+      <c r="I60" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2543,8 +2546,8 @@
       <c r="H61" s="1" t="n">
         <v>0.113</v>
       </c>
-      <c r="I61" s="1" t="n">
-        <v>1</v>
+      <c r="I61" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2572,8 +2575,8 @@
       <c r="H62" s="1" t="n">
         <v>0.0775</v>
       </c>
-      <c r="I62" s="1" t="n">
-        <v>1</v>
+      <c r="I62" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2601,8 +2604,8 @@
       <c r="H63" s="1" t="n">
         <v>0.1896</v>
       </c>
-      <c r="I63" s="1" t="n">
-        <v>1</v>
+      <c r="I63" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2630,8 +2633,8 @@
       <c r="H64" s="1" t="n">
         <v>0.3651</v>
       </c>
-      <c r="I64" s="1" t="n">
-        <v>1</v>
+      <c r="I64" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2659,8 +2662,8 @@
       <c r="H65" s="1" t="n">
         <v>0.2267</v>
       </c>
-      <c r="I65" s="1" t="n">
-        <v>1</v>
+      <c r="I65" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2688,8 +2691,8 @@
       <c r="H66" s="1" t="n">
         <v>0.0604</v>
       </c>
-      <c r="I66" s="1" t="n">
-        <v>1</v>
+      <c r="I66" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,8 +2720,8 @@
       <c r="H67" s="1" t="n">
         <v>0.1878</v>
       </c>
-      <c r="I67" s="1" t="n">
-        <v>1</v>
+      <c r="I67" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,8 +2749,8 @@
       <c r="H68" s="1" t="n">
         <v>0.0898</v>
       </c>
-      <c r="I68" s="1" t="n">
-        <v>1</v>
+      <c r="I68" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2775,8 +2778,8 @@
       <c r="H69" s="1" t="n">
         <v>0.1235</v>
       </c>
-      <c r="I69" s="1" t="n">
-        <v>1</v>
+      <c r="I69" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2804,8 +2807,8 @@
       <c r="H70" s="1" t="n">
         <v>0.3767</v>
       </c>
-      <c r="I70" s="1" t="n">
-        <v>1</v>
+      <c r="I70" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2833,8 +2836,8 @@
       <c r="H71" s="1" t="n">
         <v>0.1257</v>
       </c>
-      <c r="I71" s="1" t="n">
-        <v>1</v>
+      <c r="I71" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2862,8 +2865,8 @@
       <c r="H72" s="1" t="n">
         <v>0.1012</v>
       </c>
-      <c r="I72" s="1" t="n">
-        <v>1</v>
+      <c r="I72" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,8 +2894,8 @@
       <c r="H73" s="1" t="n">
         <v>0.3471</v>
       </c>
-      <c r="I73" s="1" t="n">
-        <v>1</v>
+      <c r="I73" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2920,8 +2923,8 @@
       <c r="H74" s="1" t="n">
         <v>0.2093</v>
       </c>
-      <c r="I74" s="1" t="n">
-        <v>1</v>
+      <c r="I74" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2949,8 +2952,8 @@
       <c r="H75" s="1" t="n">
         <v>0.2126</v>
       </c>
-      <c r="I75" s="1" t="n">
-        <v>1</v>
+      <c r="I75" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2978,8 +2981,8 @@
       <c r="H76" s="1" t="n">
         <v>0.1338</v>
       </c>
-      <c r="I76" s="1" t="n">
-        <v>1</v>
+      <c r="I76" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3007,7 +3010,7 @@
       <c r="H77" s="1" t="n">
         <v>0.0071</v>
       </c>
-      <c r="I77" s="1" t="n">
+      <c r="I77" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3036,8 +3039,8 @@
       <c r="H78" s="1" t="n">
         <v>0.0072</v>
       </c>
-      <c r="I78" s="1" t="n">
-        <v>0</v>
+      <c r="I78" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3065,8 +3068,8 @@
       <c r="H79" s="1" t="n">
         <v>0.0569</v>
       </c>
-      <c r="I79" s="1" t="n">
-        <v>0</v>
+      <c r="I79" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3094,8 +3097,8 @@
       <c r="H80" s="1" t="n">
         <v>0.0335</v>
       </c>
-      <c r="I80" s="1" t="n">
-        <v>0</v>
+      <c r="I80" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3123,7 +3126,7 @@
       <c r="H81" s="1" t="n">
         <v>0.0551</v>
       </c>
-      <c r="I81" s="1" t="n">
+      <c r="I81" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3152,8 +3155,8 @@
       <c r="H82" s="1" t="n">
         <v>0.0582</v>
       </c>
-      <c r="I82" s="1" t="n">
-        <v>1</v>
+      <c r="I82" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3181,8 +3184,8 @@
       <c r="H83" s="1" t="n">
         <v>0.0919</v>
       </c>
-      <c r="I83" s="1" t="n">
-        <v>1</v>
+      <c r="I83" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3210,8 +3213,8 @@
       <c r="H84" s="1" t="n">
         <v>0.1962</v>
       </c>
-      <c r="I84" s="1" t="n">
-        <v>1</v>
+      <c r="I84" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3239,8 +3242,8 @@
       <c r="H85" s="1" t="n">
         <v>0.1931</v>
       </c>
-      <c r="I85" s="1" t="n">
-        <v>1</v>
+      <c r="I85" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3268,8 +3271,8 @@
       <c r="H86" s="1" t="n">
         <v>0.0469</v>
       </c>
-      <c r="I86" s="1" t="n">
-        <v>1</v>
+      <c r="I86" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3297,8 +3300,8 @@
       <c r="H87" s="1" t="n">
         <v>0.1478</v>
       </c>
-      <c r="I87" s="1" t="n">
-        <v>1</v>
+      <c r="I87" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3326,8 +3329,8 @@
       <c r="H88" s="1" t="n">
         <v>0.1083</v>
       </c>
-      <c r="I88" s="1" t="n">
-        <v>1</v>
+      <c r="I88" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3355,8 +3358,8 @@
       <c r="H89" s="1" t="n">
         <v>0.2201</v>
       </c>
-      <c r="I89" s="1" t="n">
-        <v>1</v>
+      <c r="I89" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3384,8 +3387,8 @@
       <c r="H90" s="1" t="n">
         <v>0.2012</v>
       </c>
-      <c r="I90" s="1" t="n">
-        <v>1</v>
+      <c r="I90" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3413,8 +3416,8 @@
       <c r="H91" s="1" t="n">
         <v>0.2235</v>
       </c>
-      <c r="I91" s="1" t="n">
-        <v>1</v>
+      <c r="I91" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3442,8 +3445,8 @@
       <c r="H92" s="1" t="n">
         <v>0.1453</v>
       </c>
-      <c r="I92" s="1" t="n">
-        <v>1</v>
+      <c r="I92" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3471,8 +3474,8 @@
       <c r="H93" s="1" t="n">
         <v>0.1342</v>
       </c>
-      <c r="I93" s="1" t="n">
-        <v>1</v>
+      <c r="I93" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3500,8 +3503,8 @@
       <c r="H94" s="1" t="n">
         <v>0.1107</v>
       </c>
-      <c r="I94" s="1" t="n">
-        <v>1</v>
+      <c r="I94" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3529,8 +3532,8 @@
       <c r="H95" s="1" t="n">
         <v>0.1416</v>
       </c>
-      <c r="I95" s="1" t="n">
-        <v>1</v>
+      <c r="I95" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3558,8 +3561,8 @@
       <c r="H96" s="1" t="n">
         <v>0.3162</v>
       </c>
-      <c r="I96" s="1" t="n">
-        <v>1</v>
+      <c r="I96" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,8 +3590,8 @@
       <c r="H97" s="1" t="n">
         <v>0.1379</v>
       </c>
-      <c r="I97" s="1" t="n">
-        <v>1</v>
+      <c r="I97" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3616,8 +3619,8 @@
       <c r="H98" s="1" t="n">
         <v>0.2425</v>
       </c>
-      <c r="I98" s="1" t="n">
-        <v>1</v>
+      <c r="I98" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3645,8 +3648,8 @@
       <c r="H99" s="1" t="n">
         <v>0.1371</v>
       </c>
-      <c r="I99" s="1" t="n">
-        <v>1</v>
+      <c r="I99" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,8 +3677,8 @@
       <c r="H100" s="1" t="n">
         <v>0.2218</v>
       </c>
-      <c r="I100" s="1" t="n">
-        <v>1</v>
+      <c r="I100" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,8 +3706,8 @@
       <c r="H101" s="1" t="n">
         <v>0.024</v>
       </c>
-      <c r="I101" s="1" t="n">
-        <v>1</v>
+      <c r="I101" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3732,7 +3735,7 @@
       <c r="H102" s="1" t="n">
         <v>0.0073</v>
       </c>
-      <c r="I102" s="1" t="n">
+      <c r="I102" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3761,8 +3764,8 @@
       <c r="H103" s="1" t="n">
         <v>0.039</v>
       </c>
-      <c r="I103" s="1" t="n">
-        <v>0</v>
+      <c r="I103" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3790,8 +3793,8 @@
       <c r="H104" s="1" t="n">
         <v>0.0351</v>
       </c>
-      <c r="I104" s="1" t="n">
-        <v>0</v>
+      <c r="I104" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3819,8 +3822,8 @@
       <c r="H105" s="1" t="n">
         <v>0.0295</v>
       </c>
-      <c r="I105" s="1" t="n">
-        <v>0</v>
+      <c r="I105" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,7 +3851,7 @@
       <c r="H106" s="1" t="n">
         <v>0.0344</v>
       </c>
-      <c r="I106" s="1" t="n">
+      <c r="I106" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3877,8 +3880,8 @@
       <c r="H107" s="1" t="n">
         <v>0.0971</v>
       </c>
-      <c r="I107" s="1" t="n">
-        <v>1</v>
+      <c r="I107" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,8 +3909,8 @@
       <c r="H108" s="1" t="n">
         <v>0.0641</v>
       </c>
-      <c r="I108" s="1" t="n">
-        <v>1</v>
+      <c r="I108" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3935,8 +3938,8 @@
       <c r="H109" s="1" t="n">
         <v>0.1118</v>
       </c>
-      <c r="I109" s="1" t="n">
-        <v>1</v>
+      <c r="I109" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3964,8 +3967,8 @@
       <c r="H110" s="1" t="n">
         <v>0.0785</v>
       </c>
-      <c r="I110" s="1" t="n">
-        <v>1</v>
+      <c r="I110" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3993,8 +3996,8 @@
       <c r="H111" s="1" t="n">
         <v>0.1225</v>
       </c>
-      <c r="I111" s="1" t="n">
-        <v>1</v>
+      <c r="I111" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4022,8 +4025,8 @@
       <c r="H112" s="1" t="n">
         <v>0.1531</v>
       </c>
-      <c r="I112" s="1" t="n">
-        <v>1</v>
+      <c r="I112" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4051,8 +4054,8 @@
       <c r="H113" s="1" t="n">
         <v>0.2107</v>
       </c>
-      <c r="I113" s="1" t="n">
-        <v>1</v>
+      <c r="I113" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4080,8 +4083,8 @@
       <c r="H114" s="1" t="n">
         <v>0.259</v>
       </c>
-      <c r="I114" s="1" t="n">
-        <v>1</v>
+      <c r="I114" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,8 +4112,8 @@
       <c r="H115" s="1" t="n">
         <v>0.5903</v>
       </c>
-      <c r="I115" s="1" t="n">
-        <v>1</v>
+      <c r="I115" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4138,8 +4141,8 @@
       <c r="H116" s="1" t="n">
         <v>0.3177</v>
       </c>
-      <c r="I116" s="1" t="n">
-        <v>1</v>
+      <c r="I116" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4167,8 +4170,8 @@
       <c r="H117" s="1" t="n">
         <v>0.322</v>
       </c>
-      <c r="I117" s="1" t="n">
-        <v>1</v>
+      <c r="I117" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4196,8 +4199,8 @@
       <c r="H118" s="1" t="n">
         <v>0.1332</v>
       </c>
-      <c r="I118" s="1" t="n">
-        <v>1</v>
+      <c r="I118" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4225,8 +4228,8 @@
       <c r="H119" s="1" t="n">
         <v>0.1843</v>
       </c>
-      <c r="I119" s="1" t="n">
-        <v>1</v>
+      <c r="I119" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4254,8 +4257,8 @@
       <c r="H120" s="1" t="n">
         <v>0.1043</v>
       </c>
-      <c r="I120" s="1" t="n">
-        <v>1</v>
+      <c r="I120" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4283,8 +4286,8 @@
       <c r="H121" s="1" t="n">
         <v>0.1688</v>
       </c>
-      <c r="I121" s="1" t="n">
-        <v>1</v>
+      <c r="I121" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4312,8 +4315,8 @@
       <c r="H122" s="1" t="n">
         <v>0.1397</v>
       </c>
-      <c r="I122" s="1" t="n">
-        <v>1</v>
+      <c r="I122" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4341,8 +4344,8 @@
       <c r="H123" s="1" t="n">
         <v>0.217</v>
       </c>
-      <c r="I123" s="1" t="n">
-        <v>1</v>
+      <c r="I123" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4370,8 +4373,8 @@
       <c r="H124" s="1" t="n">
         <v>0.3731</v>
       </c>
-      <c r="I124" s="1" t="n">
-        <v>1</v>
+      <c r="I124" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4399,8 +4402,8 @@
       <c r="H125" s="1" t="n">
         <v>0.808</v>
       </c>
-      <c r="I125" s="1" t="n">
-        <v>1</v>
+      <c r="I125" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4428,8 +4431,8 @@
       <c r="H126" s="1" t="n">
         <v>0.0305</v>
       </c>
-      <c r="I126" s="1" t="n">
-        <v>1</v>
+      <c r="I126" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4457,7 +4460,7 @@
       <c r="H127" s="1" t="n">
         <v>0.0033</v>
       </c>
-      <c r="I127" s="1" t="n">
+      <c r="I127" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4486,8 +4489,8 @@
       <c r="H128" s="1" t="n">
         <v>0.0215</v>
       </c>
-      <c r="I128" s="1" t="n">
-        <v>0</v>
+      <c r="I128" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4515,8 +4518,8 @@
       <c r="H129" s="1" t="n">
         <v>0.0578</v>
       </c>
-      <c r="I129" s="1" t="n">
-        <v>0</v>
+      <c r="I129" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4544,8 +4547,8 @@
       <c r="H130" s="1" t="n">
         <v>0.0413</v>
       </c>
-      <c r="I130" s="1" t="n">
-        <v>0</v>
+      <c r="I130" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4573,8 +4576,8 @@
       <c r="H131" s="1" t="n">
         <v>0.0594</v>
       </c>
-      <c r="I131" s="1" t="n">
-        <v>0</v>
+      <c r="I131" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4602,8 +4605,8 @@
       <c r="H132" s="1" t="n">
         <v>0.0407</v>
       </c>
-      <c r="I132" s="1" t="n">
-        <v>1</v>
+      <c r="I132" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4631,8 +4634,8 @@
       <c r="H133" s="1" t="n">
         <v>0.2223</v>
       </c>
-      <c r="I133" s="1" t="n">
-        <v>1</v>
+      <c r="I133" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4660,8 +4663,8 @@
       <c r="H134" s="1" t="n">
         <v>0.1631</v>
       </c>
-      <c r="I134" s="1" t="n">
-        <v>1</v>
+      <c r="I134" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4689,8 +4692,8 @@
       <c r="H135" s="1" t="n">
         <v>0.0919</v>
       </c>
-      <c r="I135" s="1" t="n">
-        <v>1</v>
+      <c r="I135" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4718,8 +4721,8 @@
       <c r="H136" s="1" t="n">
         <v>0.1212</v>
       </c>
-      <c r="I136" s="1" t="n">
-        <v>1</v>
+      <c r="I136" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4747,8 +4750,8 @@
       <c r="H137" s="1" t="n">
         <v>0.1618</v>
       </c>
-      <c r="I137" s="1" t="n">
-        <v>1</v>
+      <c r="I137" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4776,8 +4779,8 @@
       <c r="H138" s="1" t="n">
         <v>0.3568</v>
       </c>
-      <c r="I138" s="1" t="n">
-        <v>1</v>
+      <c r="I138" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4805,8 +4808,8 @@
       <c r="H139" s="1" t="n">
         <v>0.3322</v>
       </c>
-      <c r="I139" s="1" t="n">
-        <v>1</v>
+      <c r="I139" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4834,8 +4837,8 @@
       <c r="H140" s="1" t="n">
         <v>0.0685</v>
       </c>
-      <c r="I140" s="1" t="n">
-        <v>1</v>
+      <c r="I140" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4863,8 +4866,8 @@
       <c r="H141" s="1" t="n">
         <v>0.1018</v>
       </c>
-      <c r="I141" s="1" t="n">
-        <v>1</v>
+      <c r="I141" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4892,8 +4895,8 @@
       <c r="H142" s="1" t="n">
         <v>0.1557</v>
       </c>
-      <c r="I142" s="1" t="n">
-        <v>1</v>
+      <c r="I142" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4921,8 +4924,8 @@
       <c r="H143" s="1" t="n">
         <v>0.2422</v>
       </c>
-      <c r="I143" s="1" t="n">
-        <v>1</v>
+      <c r="I143" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4950,8 +4953,8 @@
       <c r="H144" s="1" t="n">
         <v>0.1429</v>
       </c>
-      <c r="I144" s="1" t="n">
-        <v>1</v>
+      <c r="I144" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4979,8 +4982,8 @@
       <c r="H145" s="1" t="n">
         <v>0.1964</v>
       </c>
-      <c r="I145" s="1" t="n">
-        <v>1</v>
+      <c r="I145" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5008,8 +5011,8 @@
       <c r="H146" s="1" t="n">
         <v>0.1322</v>
       </c>
-      <c r="I146" s="1" t="n">
-        <v>1</v>
+      <c r="I146" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,8 +5040,8 @@
       <c r="H147" s="1" t="n">
         <v>0.1181</v>
       </c>
-      <c r="I147" s="1" t="n">
-        <v>1</v>
+      <c r="I147" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5066,8 +5069,8 @@
       <c r="H148" s="1" t="n">
         <v>0.8833</v>
       </c>
-      <c r="I148" s="1" t="n">
-        <v>1</v>
+      <c r="I148" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5095,8 +5098,8 @@
       <c r="H149" s="1" t="n">
         <v>0.1092</v>
       </c>
-      <c r="I149" s="1" t="n">
-        <v>1</v>
+      <c r="I149" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,8 +5127,8 @@
       <c r="H150" s="1" t="n">
         <v>0.2869</v>
       </c>
-      <c r="I150" s="1" t="n">
-        <v>1</v>
+      <c r="I150" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5153,8 +5156,8 @@
       <c r="H151" s="1" t="n">
         <v>0.222</v>
       </c>
-      <c r="I151" s="1" t="n">
-        <v>1</v>
+      <c r="I151" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5182,7 +5185,7 @@
       <c r="H152" s="1" t="n">
         <v>0.0027</v>
       </c>
-      <c r="I152" s="1" t="n">
+      <c r="I152" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5211,8 +5214,8 @@
       <c r="H153" s="1" t="n">
         <v>0.0024</v>
       </c>
-      <c r="I153" s="1" t="n">
-        <v>0</v>
+      <c r="I153" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5240,8 +5243,8 @@
       <c r="H154" s="1" t="n">
         <v>0.0029</v>
       </c>
-      <c r="I154" s="1" t="n">
-        <v>0</v>
+      <c r="I154" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5269,8 +5272,8 @@
       <c r="H155" s="1" t="n">
         <v>0.0127</v>
       </c>
-      <c r="I155" s="1" t="n">
-        <v>0</v>
+      <c r="I155" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5298,8 +5301,8 @@
       <c r="H156" s="1" t="n">
         <v>0.0686</v>
       </c>
-      <c r="I156" s="1" t="n">
-        <v>1</v>
+      <c r="I156" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5327,8 +5330,8 @@
       <c r="H157" s="1" t="n">
         <v>0.1057</v>
       </c>
-      <c r="I157" s="1" t="n">
-        <v>1</v>
+      <c r="I157" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5356,8 +5359,8 @@
       <c r="H158" s="1" t="n">
         <v>0.2427</v>
       </c>
-      <c r="I158" s="1" t="n">
-        <v>1</v>
+      <c r="I158" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,8 +5388,8 @@
       <c r="H159" s="1" t="n">
         <v>0.0919</v>
       </c>
-      <c r="I159" s="1" t="n">
-        <v>1</v>
+      <c r="I159" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5414,8 +5417,8 @@
       <c r="H160" s="1" t="n">
         <v>0.079</v>
       </c>
-      <c r="I160" s="1" t="n">
-        <v>1</v>
+      <c r="I160" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5443,8 +5446,8 @@
       <c r="H161" s="1" t="n">
         <v>0.1879</v>
       </c>
-      <c r="I161" s="1" t="n">
-        <v>1</v>
+      <c r="I161" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5472,8 +5475,8 @@
       <c r="H162" s="1" t="n">
         <v>0.0933</v>
       </c>
-      <c r="I162" s="1" t="n">
-        <v>1</v>
+      <c r="I162" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5501,8 +5504,8 @@
       <c r="H163" s="1" t="n">
         <v>0.1314</v>
       </c>
-      <c r="I163" s="1" t="n">
-        <v>1</v>
+      <c r="I163" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5530,8 +5533,8 @@
       <c r="H164" s="1" t="n">
         <v>0.2584</v>
       </c>
-      <c r="I164" s="1" t="n">
-        <v>1</v>
+      <c r="I164" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5559,8 +5562,8 @@
       <c r="H165" s="1" t="n">
         <v>0.1179</v>
       </c>
-      <c r="I165" s="1" t="n">
-        <v>1</v>
+      <c r="I165" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5588,8 +5591,8 @@
       <c r="H166" s="1" t="n">
         <v>0.1948</v>
       </c>
-      <c r="I166" s="1" t="n">
-        <v>1</v>
+      <c r="I166" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5617,8 +5620,8 @@
       <c r="H167" s="1" t="n">
         <v>0.1348</v>
       </c>
-      <c r="I167" s="1" t="n">
-        <v>1</v>
+      <c r="I167" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5646,8 +5649,8 @@
       <c r="H168" s="1" t="n">
         <v>0.2719</v>
       </c>
-      <c r="I168" s="1" t="n">
-        <v>1</v>
+      <c r="I168" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5675,8 +5678,8 @@
       <c r="H169" s="1" t="n">
         <v>0.1343</v>
       </c>
-      <c r="I169" s="1" t="n">
-        <v>1</v>
+      <c r="I169" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5704,8 +5707,8 @@
       <c r="H170" s="1" t="n">
         <v>0.1741</v>
       </c>
-      <c r="I170" s="1" t="n">
-        <v>1</v>
+      <c r="I170" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5733,8 +5736,8 @@
       <c r="H171" s="1" t="n">
         <v>0.4131</v>
       </c>
-      <c r="I171" s="1" t="n">
-        <v>1</v>
+      <c r="I171" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5762,8 +5765,8 @@
       <c r="H172" s="1" t="n">
         <v>0.1593</v>
       </c>
-      <c r="I172" s="1" t="n">
-        <v>1</v>
+      <c r="I172" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5791,8 +5794,8 @@
       <c r="H173" s="1" t="n">
         <v>0.4367</v>
       </c>
-      <c r="I173" s="1" t="n">
-        <v>1</v>
+      <c r="I173" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5820,8 +5823,8 @@
       <c r="H174" s="1" t="n">
         <v>0.8056</v>
       </c>
-      <c r="I174" s="1" t="n">
-        <v>1</v>
+      <c r="I174" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5849,8 +5852,8 @@
       <c r="H175" s="1" t="n">
         <v>0.2069</v>
       </c>
-      <c r="I175" s="1" t="n">
-        <v>1</v>
+      <c r="I175" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5878,8 +5881,8 @@
       <c r="H176" s="1" t="n">
         <v>0.0033</v>
       </c>
-      <c r="I176" s="1" t="n">
-        <v>0</v>
+      <c r="I176" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5907,8 +5910,8 @@
       <c r="H177" s="1" t="n">
         <v>0.0081</v>
       </c>
-      <c r="I177" s="1" t="n">
-        <v>0</v>
+      <c r="I177" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5936,8 +5939,8 @@
       <c r="H178" s="1" t="n">
         <v>0.0092</v>
       </c>
-      <c r="I178" s="1" t="n">
-        <v>0</v>
+      <c r="I178" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5965,8 +5968,8 @@
       <c r="H179" s="1" t="n">
         <v>0.033</v>
       </c>
-      <c r="I179" s="1" t="n">
-        <v>0</v>
+      <c r="I179" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5994,7 +5997,7 @@
       <c r="H180" s="1" t="n">
         <v>0.1785</v>
       </c>
-      <c r="I180" s="1" t="n">
+      <c r="I180" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6023,8 +6026,8 @@
       <c r="H181" s="1" t="n">
         <v>0.1309</v>
       </c>
-      <c r="I181" s="1" t="n">
-        <v>1</v>
+      <c r="I181" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6052,8 +6055,8 @@
       <c r="H182" s="1" t="n">
         <v>0.1327</v>
       </c>
-      <c r="I182" s="1" t="n">
-        <v>1</v>
+      <c r="I182" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6081,8 +6084,8 @@
       <c r="H183" s="1" t="n">
         <v>0.1925</v>
       </c>
-      <c r="I183" s="1" t="n">
-        <v>1</v>
+      <c r="I183" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6110,8 +6113,8 @@
       <c r="H184" s="1" t="n">
         <v>0.1089</v>
       </c>
-      <c r="I184" s="1" t="n">
-        <v>1</v>
+      <c r="I184" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6139,8 +6142,8 @@
       <c r="H185" s="1" t="n">
         <v>0.2568</v>
       </c>
-      <c r="I185" s="1" t="n">
-        <v>1</v>
+      <c r="I185" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6168,8 +6171,8 @@
       <c r="H186" s="1" t="n">
         <v>0.0794</v>
       </c>
-      <c r="I186" s="1" t="n">
-        <v>1</v>
+      <c r="I186" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6197,8 +6200,8 @@
       <c r="H187" s="1" t="n">
         <v>0.1548</v>
       </c>
-      <c r="I187" s="1" t="n">
-        <v>1</v>
+      <c r="I187" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6226,8 +6229,8 @@
       <c r="H188" s="1" t="n">
         <v>0.284</v>
       </c>
-      <c r="I188" s="1" t="n">
-        <v>1</v>
+      <c r="I188" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6255,8 +6258,8 @@
       <c r="H189" s="1" t="n">
         <v>0.3891</v>
       </c>
-      <c r="I189" s="1" t="n">
-        <v>1</v>
+      <c r="I189" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6284,8 +6287,8 @@
       <c r="H190" s="1" t="n">
         <v>0.2379</v>
       </c>
-      <c r="I190" s="1" t="n">
-        <v>1</v>
+      <c r="I190" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6313,8 +6316,8 @@
       <c r="H191" s="1" t="n">
         <v>0.2096</v>
       </c>
-      <c r="I191" s="1" t="n">
-        <v>1</v>
+      <c r="I191" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6342,8 +6345,8 @@
       <c r="H192" s="1" t="n">
         <v>0.0186</v>
       </c>
-      <c r="I192" s="1" t="n">
-        <v>1</v>
+      <c r="I192" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6371,8 +6374,8 @@
       <c r="H193" s="1" t="n">
         <v>0.1109</v>
       </c>
-      <c r="I193" s="1" t="n">
-        <v>0</v>
+      <c r="I193" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6400,8 +6403,8 @@
       <c r="H194" s="1" t="n">
         <v>0.0495</v>
       </c>
-      <c r="I194" s="1" t="n">
-        <v>0</v>
+      <c r="I194" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6429,8 +6432,8 @@
       <c r="H195" s="1" t="n">
         <v>0.065</v>
       </c>
-      <c r="I195" s="1" t="n">
-        <v>0</v>
+      <c r="I195" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6458,8 +6461,8 @@
       <c r="H196" s="1" t="n">
         <v>0.0691</v>
       </c>
-      <c r="I196" s="1" t="n">
-        <v>0</v>
+      <c r="I196" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6487,8 +6490,8 @@
       <c r="H197" s="1" t="n">
         <v>0.0958</v>
       </c>
-      <c r="I197" s="1" t="n">
-        <v>1</v>
+      <c r="I197" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6516,8 +6519,8 @@
       <c r="H198" s="1" t="n">
         <v>0.0937</v>
       </c>
-      <c r="I198" s="1" t="n">
-        <v>1</v>
+      <c r="I198" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6545,8 +6548,8 @@
       <c r="H199" s="1" t="n">
         <v>0.1093</v>
       </c>
-      <c r="I199" s="1" t="n">
-        <v>1</v>
+      <c r="I199" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6574,8 +6577,8 @@
       <c r="H200" s="1" t="n">
         <v>0.0907</v>
       </c>
-      <c r="I200" s="1" t="n">
-        <v>1</v>
+      <c r="I200" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6603,8 +6606,8 @@
       <c r="H201" s="1" t="n">
         <v>0.199</v>
       </c>
-      <c r="I201" s="1" t="n">
-        <v>1</v>
+      <c r="I201" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6632,8 +6635,8 @@
       <c r="H202" s="1" t="n">
         <v>0.0807</v>
       </c>
-      <c r="I202" s="1" t="n">
-        <v>1</v>
+      <c r="I202" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6661,8 +6664,8 @@
       <c r="H203" s="1" t="n">
         <v>0.0394</v>
       </c>
-      <c r="I203" s="1" t="n">
-        <v>1</v>
+      <c r="I203" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>